<commit_message>
Added more functionality to semantic analysis
</commit_message>
<xml_diff>
--- a/chybove_hlasenia.xlsx
+++ b/chybove_hlasenia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marko\Documents\VUT FIT\ifj\proj\ifj-projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C51D90-DA2A-4A81-A7AA-C675166AE6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B3ABBF0-6AD6-4647-A2C9-F4D62DD2897B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{3659E002-BE5E-4071-95AA-5C6DB9B812AC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>Popis</t>
   </si>
@@ -361,14 +361,6 @@
   <si>
     <t>Žádný z operátorů nelze aplikovat na řezy
  nebo řetězcové literály.</t>
-  </si>
-  <si>
-    <t>Bez rozšíření
-BOOLTHEN není s výsledkem porovnání (pravdivostní hodnota) možné dále pracovat a
-lze jej využít pouze u podmínek příkazů if a while</t>
-  </si>
-  <si>
-    <t>TODO</t>
   </si>
   <si>
     <t>V případě, že příkaz volání
@@ -869,7 +861,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -919,7 +911,7 @@
     </row>
     <row r="8" spans="1:5" ht="111.9" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A8" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B8" s="2">
         <v>5</v>
@@ -1050,6 +1042,9 @@
       <c r="B17" s="2">
         <v>7</v>
       </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
       <c r="D17" s="1" t="s">
         <v>38</v>
       </c>
@@ -1061,13 +1056,16 @@
       <c r="B18" s="2">
         <v>8</v>
       </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
       <c r="D18" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="192" x14ac:dyDescent="0.7">
       <c r="A19" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B19" s="2">
         <v>4</v>
@@ -1212,27 +1210,30 @@
     </row>
     <row r="30" spans="1:4" ht="60.9" x14ac:dyDescent="0.7">
       <c r="A30" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B30" s="2">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60.9" x14ac:dyDescent="0.7">
       <c r="A31" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B31" s="2">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60.9" x14ac:dyDescent="0.7">
@@ -1242,25 +1243,15 @@
       <c r="B32" s="2">
         <v>5</v>
       </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
       <c r="D32" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="60.9" x14ac:dyDescent="0.7">
-      <c r="A33" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B33" s="2">
-        <v>5</v>
-      </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.7">
+      <c r="A34" s="1"/>
       <c r="D34" s="1"/>
     </row>
   </sheetData>

</xml_diff>